<commit_message>
adda pri men må testets
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEB0EB9-ED56-463C-A2D0-3C524DBED300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C60773-F857-43D2-8084-4B0102BE07ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site 1 (HUB)" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="43">
   <si>
     <t>site</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t>tunnel 30</t>
+  </si>
+  <si>
+    <t>antall-res</t>
+  </si>
+  <si>
+    <t>pri-1-10</t>
   </si>
 </sst>
 </file>
@@ -292,7 +298,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="144">
+  <dxfs count="154">
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
@@ -300,12 +312,174 @@
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -414,124 +588,40 @@
       <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" justifyLastLine="0" shrinkToFit="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -1149,127 +1239,103 @@
         </bottom>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="16">
     <tableStyle name="Site 1 (HUB)-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="140"/>
-      <tableStyleElement type="headerRow" dxfId="143"/>
-      <tableStyleElement type="firstRowStripe" dxfId="142"/>
-      <tableStyleElement type="secondRowStripe" dxfId="141"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="153"/>
+      <tableStyleElement type="headerRow" dxfId="152"/>
+      <tableStyleElement type="firstRowStripe" dxfId="151"/>
+      <tableStyleElement type="secondRowStripe" dxfId="150"/>
     </tableStyle>
     <tableStyle name="Site 3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="136"/>
-      <tableStyleElement type="headerRow" dxfId="139"/>
-      <tableStyleElement type="firstRowStripe" dxfId="138"/>
-      <tableStyleElement type="secondRowStripe" dxfId="137"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="149"/>
+      <tableStyleElement type="headerRow" dxfId="148"/>
+      <tableStyleElement type="firstRowStripe" dxfId="147"/>
+      <tableStyleElement type="secondRowStripe" dxfId="146"/>
     </tableStyle>
     <tableStyle name="Site 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="132"/>
-      <tableStyleElement type="headerRow" dxfId="135"/>
-      <tableStyleElement type="firstRowStripe" dxfId="134"/>
-      <tableStyleElement type="secondRowStripe" dxfId="133"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="145"/>
+      <tableStyleElement type="headerRow" dxfId="144"/>
+      <tableStyleElement type="firstRowStripe" dxfId="143"/>
+      <tableStyleElement type="secondRowStripe" dxfId="142"/>
     </tableStyle>
     <tableStyle name="Site 4-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="128"/>
-      <tableStyleElement type="headerRow" dxfId="131"/>
-      <tableStyleElement type="firstRowStripe" dxfId="130"/>
-      <tableStyleElement type="secondRowStripe" dxfId="129"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="141"/>
+      <tableStyleElement type="headerRow" dxfId="140"/>
+      <tableStyleElement type="firstRowStripe" dxfId="139"/>
+      <tableStyleElement type="secondRowStripe" dxfId="138"/>
     </tableStyle>
     <tableStyle name="Site 3-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="124"/>
-      <tableStyleElement type="headerRow" dxfId="127"/>
-      <tableStyleElement type="firstRowStripe" dxfId="126"/>
-      <tableStyleElement type="secondRowStripe" dxfId="125"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="137"/>
+      <tableStyleElement type="headerRow" dxfId="136"/>
+      <tableStyleElement type="firstRowStripe" dxfId="135"/>
+      <tableStyleElement type="secondRowStripe" dxfId="134"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="120"/>
-      <tableStyleElement type="headerRow" dxfId="123"/>
-      <tableStyleElement type="firstRowStripe" dxfId="122"/>
-      <tableStyleElement type="secondRowStripe" dxfId="121"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="133"/>
+      <tableStyleElement type="headerRow" dxfId="132"/>
+      <tableStyleElement type="firstRowStripe" dxfId="131"/>
+      <tableStyleElement type="secondRowStripe" dxfId="130"/>
     </tableStyle>
     <tableStyle name="Site 2-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="116"/>
-      <tableStyleElement type="headerRow" dxfId="119"/>
-      <tableStyleElement type="firstRowStripe" dxfId="118"/>
-      <tableStyleElement type="secondRowStripe" dxfId="117"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="129"/>
+      <tableStyleElement type="headerRow" dxfId="128"/>
+      <tableStyleElement type="firstRowStripe" dxfId="127"/>
+      <tableStyleElement type="secondRowStripe" dxfId="126"/>
     </tableStyle>
     <tableStyle name="Site 3-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="112"/>
-      <tableStyleElement type="headerRow" dxfId="115"/>
-      <tableStyleElement type="firstRowStripe" dxfId="114"/>
-      <tableStyleElement type="secondRowStripe" dxfId="113"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="125"/>
+      <tableStyleElement type="headerRow" dxfId="124"/>
+      <tableStyleElement type="firstRowStripe" dxfId="123"/>
+      <tableStyleElement type="secondRowStripe" dxfId="122"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF08000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="108"/>
-      <tableStyleElement type="headerRow" dxfId="111"/>
-      <tableStyleElement type="firstRowStripe" dxfId="110"/>
-      <tableStyleElement type="secondRowStripe" dxfId="109"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="121"/>
+      <tableStyleElement type="headerRow" dxfId="120"/>
+      <tableStyleElement type="firstRowStripe" dxfId="119"/>
+      <tableStyleElement type="secondRowStripe" dxfId="118"/>
     </tableStyle>
     <tableStyle name="Site 4-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF09000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="104"/>
-      <tableStyleElement type="headerRow" dxfId="107"/>
-      <tableStyleElement type="firstRowStripe" dxfId="106"/>
-      <tableStyleElement type="secondRowStripe" dxfId="105"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="117"/>
+      <tableStyleElement type="headerRow" dxfId="116"/>
+      <tableStyleElement type="firstRowStripe" dxfId="115"/>
+      <tableStyleElement type="secondRowStripe" dxfId="114"/>
     </tableStyle>
     <tableStyle name="Site 3-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0A000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="100"/>
-      <tableStyleElement type="headerRow" dxfId="103"/>
-      <tableStyleElement type="firstRowStripe" dxfId="102"/>
-      <tableStyleElement type="secondRowStripe" dxfId="101"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="113"/>
+      <tableStyleElement type="headerRow" dxfId="112"/>
+      <tableStyleElement type="firstRowStripe" dxfId="111"/>
+      <tableStyleElement type="secondRowStripe" dxfId="110"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0B000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="96"/>
-      <tableStyleElement type="headerRow" dxfId="99"/>
-      <tableStyleElement type="firstRowStripe" dxfId="98"/>
-      <tableStyleElement type="secondRowStripe" dxfId="97"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="109"/>
+      <tableStyleElement type="headerRow" dxfId="108"/>
+      <tableStyleElement type="firstRowStripe" dxfId="107"/>
+      <tableStyleElement type="secondRowStripe" dxfId="106"/>
     </tableStyle>
     <tableStyle name="Site 2-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0C000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="92"/>
-      <tableStyleElement type="headerRow" dxfId="95"/>
-      <tableStyleElement type="firstRowStripe" dxfId="94"/>
-      <tableStyleElement type="secondRowStripe" dxfId="93"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="105"/>
+      <tableStyleElement type="headerRow" dxfId="104"/>
+      <tableStyleElement type="firstRowStripe" dxfId="103"/>
+      <tableStyleElement type="secondRowStripe" dxfId="102"/>
     </tableStyle>
     <tableStyle name="Site 4-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0D000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="88"/>
-      <tableStyleElement type="headerRow" dxfId="91"/>
-      <tableStyleElement type="firstRowStripe" dxfId="90"/>
-      <tableStyleElement type="secondRowStripe" dxfId="89"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="101"/>
+      <tableStyleElement type="headerRow" dxfId="100"/>
+      <tableStyleElement type="firstRowStripe" dxfId="99"/>
+      <tableStyleElement type="secondRowStripe" dxfId="98"/>
     </tableStyle>
     <tableStyle name="Site 2-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0E000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="84"/>
-      <tableStyleElement type="headerRow" dxfId="87"/>
-      <tableStyleElement type="firstRowStripe" dxfId="86"/>
-      <tableStyleElement type="secondRowStripe" dxfId="85"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="97"/>
+      <tableStyleElement type="headerRow" dxfId="96"/>
+      <tableStyleElement type="firstRowStripe" dxfId="95"/>
+      <tableStyleElement type="secondRowStripe" dxfId="94"/>
     </tableStyle>
     <tableStyle name="Site 4-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0F000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="80"/>
-      <tableStyleElement type="headerRow" dxfId="83"/>
-      <tableStyleElement type="firstRowStripe" dxfId="82"/>
-      <tableStyleElement type="secondRowStripe" dxfId="81"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="93"/>
+      <tableStyleElement type="headerRow" dxfId="92"/>
+      <tableStyleElement type="firstRowStripe" dxfId="91"/>
+      <tableStyleElement type="secondRowStripe" dxfId="90"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1298,114 +1364,118 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell10" displayName="Tabell10" ref="A4:H7" headerRowDxfId="22" dataDxfId="20" totalsRowDxfId="21">
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="vrf" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="vlan" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="interface" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="nett id" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="gateway" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="mask" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="address min" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0900-000008000000}" name="address max" dataDxfId="23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell10" displayName="Tabell10" ref="A4:J7" headerRowDxfId="80" dataDxfId="79" totalsRowDxfId="78">
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="vrf" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="vlan" dataDxfId="76"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="interface" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="nett id" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="gateway" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0900-000006000000}" name="mask" dataDxfId="72"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0900-000007000000}" name="address min" dataDxfId="71"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0900-000008000000}" name="address max" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{E31F8F39-D63F-4CA9-A605-F61B0B449EB7}" name="antall-res" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{872D007A-F188-416D-BDFA-5197C1FAB215}" name="pri-1-10" dataDxfId="3" totalsRowDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="Site 3-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="Tabell11" displayName="Tabell11" ref="A9:D12" headerRowDxfId="15" dataDxfId="13" totalsRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF0A000000}" name="Tabell11" displayName="Tabell11" ref="A9:D12" headerRowDxfId="69" dataDxfId="68" totalsRowDxfId="67">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="vrf" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="rt" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="loopback" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="laddr" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="vrf" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="rt" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="loopback" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="laddr" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="Site 3-style 3" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell12" displayName="Tabell12" ref="A14:J16" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell12" displayName="Tabell12" ref="A14:J16" headerRowDxfId="62" dataDxfId="61" totalsRowDxfId="60">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="tunnel id" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="vrf" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="ip address" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="mask" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="source" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="destination" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="gre mode" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="network-id" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="ipsec" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="ipsec key" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="tunnel id" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="vrf" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="ip address" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="mask" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="source" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="destination" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="gre mode" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="network-id" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="ipsec" dataDxfId="51"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="ipsec key" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="Site 3-style 4" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Tabell13" displayName="Tabell13" ref="A1:F2" headerRowDxfId="73" dataDxfId="71" totalsRowDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF0C000000}" name="Tabell13" displayName="Tabell13" ref="A1:F2" headerRowDxfId="49" dataDxfId="48" totalsRowDxfId="47">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="site" dataDxfId="79"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="intf_prefix" dataDxfId="78"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="router-id" dataDxfId="77"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="brukernavn" dataDxfId="76"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="passord" dataDxfId="75"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="vty_lines" dataDxfId="74"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0C00-000001000000}" name="site" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0C00-000002000000}" name="intf_prefix" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0C00-000003000000}" name="router-id" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0C00-000004000000}" name="brukernavn" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0C00-000005000000}" name="passord" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0C00-000006000000}" name="vty_lines" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Tabell14" displayName="Tabell14" ref="A4:H7" headerRowDxfId="62" dataDxfId="60" totalsRowDxfId="61">
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="vrf" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="vlan" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="interface" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="nett id" dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="gateway" dataDxfId="66"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="mask" dataDxfId="65"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0D00-000007000000}" name="address min" dataDxfId="64"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0D00-000008000000}" name="address max" dataDxfId="63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF0D000000}" name="Tabell14" displayName="Tabell14" ref="A4:J7" headerRowDxfId="40" dataDxfId="39" totalsRowDxfId="38">
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="vrf" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="vlan" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="interface" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="nett id" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="gateway" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="mask" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0D00-000007000000}" name="address min" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0D00-000008000000}" name="address max" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{D71A0F4B-8894-49C9-A19A-CB3D67B8C9A4}" name="antall-res" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{D72B4B49-342E-4472-A7DB-D9DD906E860B}" name="pri-1-10" dataDxfId="1" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Tabell15" displayName="Tabell15" ref="A9:D12" headerRowDxfId="55" dataDxfId="53" totalsRowDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{00000000-000C-0000-FFFF-FFFF0E000000}" name="Tabell15" displayName="Tabell15" ref="A9:D12" headerRowDxfId="29" dataDxfId="28" totalsRowDxfId="27">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="vrf" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="rt" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="loopback" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="laddr" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0E00-000001000000}" name="vrf" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0E00-000002000000}" name="rt" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0E00-000003000000}" name="loopback" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0E00-000004000000}" name="laddr" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style 3" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="Tabell16" displayName="Tabell16" ref="A14:J16" headerRowDxfId="42" dataDxfId="40" totalsRowDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{00000000-000C-0000-FFFF-FFFF0F000000}" name="Tabell16" displayName="Tabell16" ref="A14:J16" headerRowDxfId="22" dataDxfId="21" totalsRowDxfId="20">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="tunnel id" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="vrf" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="ip address" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="mask" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="source" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0F00-000006000000}" name="destination" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="gre mode" dataDxfId="46"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0F00-000008000000}" name="network-id" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0F00-000009000000}" name="ipsec" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0F00-00000A000000}" name="ipsec key" dataDxfId="43"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="tunnel id" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="vrf" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="ip address" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="mask" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="source" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0F00-000006000000}" name="destination" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="gre mode" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0F00-000008000000}" name="network-id" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0F00-000009000000}" name="ipsec" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0F00-00000A000000}" name="ipsec key" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style 4" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabell6" displayName="Tabell6" ref="A4:H7">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabell6" displayName="Tabell6" ref="A4:J7">
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="vrf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="vlan"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="interface"/>
@@ -1414,6 +1484,8 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-1-10"/>
   </tableColumns>
   <tableStyleInfo name="Site 1 (HUB)-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1464,8 +1536,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell2" displayName="Tabell2" ref="A4:H7">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell2" displayName="Tabell2" ref="A4:J7">
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="vrf"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="vlan"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="interface"/>
@@ -1474,6 +1546,8 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-1-10"/>
   </tableColumns>
   <tableStyleInfo name="Site 2-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1510,14 +1584,14 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell9" displayName="Tabell9" ref="A1:F2" headerRowDxfId="33" dataDxfId="31" totalsRowDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell9" displayName="Tabell9" ref="A1:F2" headerRowDxfId="89" dataDxfId="88" totalsRowDxfId="87">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="site" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="intf_prefix" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="router-id" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="brukernavn" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="passord" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="vty_lines" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="site" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="intf_prefix" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="router-id" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="brukernavn" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="passord" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="vty_lines" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="Site 3-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1809,6 +1883,12 @@
       <c r="H4" s="5" t="s">
         <v>17</v>
       </c>
+      <c r="I4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -1839,6 +1919,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D5,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.11.255.254")</f>
         <v>10.11.255.254</v>
       </c>
+      <c r="I5" s="6">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
@@ -1869,6 +1955,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D6,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.21.255.254")</f>
         <v>10.21.255.254</v>
       </c>
+      <c r="I6" s="6">
+        <v>10</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
@@ -1898,6 +1990,12 @@
       <c r="H7" s="6" t="str">
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D7,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.31.255.254")</f>
         <v>10.31.255.254</v>
+      </c>
+      <c r="I7" s="6">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3156,6 +3254,12 @@
       <c r="H4" s="5" t="s">
         <v>17</v>
       </c>
+      <c r="I4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -3186,6 +3290,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D5,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.12.255.254")</f>
         <v>10.12.255.254</v>
       </c>
+      <c r="I5" s="6">
+        <v>10</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
@@ -3216,6 +3326,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D6,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.22.255.254")</f>
         <v>10.22.255.254</v>
       </c>
+      <c r="I6" s="6">
+        <v>10</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
@@ -3245,6 +3361,12 @@
       <c r="H7" s="6" t="str">
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D7,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.32.255.254")</f>
         <v>10.32.255.254</v>
+      </c>
+      <c r="I7" s="6">
+        <v>10</v>
+      </c>
+      <c r="J7">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4505,8 +4627,12 @@
       <c r="H4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
+      <c r="I4" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>42</v>
+      </c>
       <c r="K4" s="11"/>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4538,8 +4664,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D5,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.13.255.254")</f>
         <v>10.13.255.254</v>
       </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
+      <c r="I5" s="16">
+        <v>10</v>
+      </c>
+      <c r="J5" s="11">
+        <v>5</v>
+      </c>
       <c r="K5" s="11"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4571,8 +4701,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D6,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.23.255.254")</f>
         <v>10.23.255.254</v>
       </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
+      <c r="I6" s="16">
+        <v>10</v>
+      </c>
+      <c r="J6" s="11">
+        <v>3</v>
+      </c>
       <c r="K6" s="11"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4604,8 +4738,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D7,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.33.255.254")</f>
         <v>10.33.255.254</v>
       </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
+      <c r="I7" s="16">
+        <v>10</v>
+      </c>
+      <c r="J7" s="11">
+        <v>10</v>
+      </c>
       <c r="K7" s="11"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5932,8 +6070,12 @@
       <c r="H4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
+      <c r="I4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
@@ -5964,8 +6106,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D5,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.14.255.254")</f>
         <v>10.14.255.254</v>
       </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
+      <c r="I5" s="6">
+        <v>10</v>
+      </c>
+      <c r="J5" s="20">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
@@ -5996,8 +6142,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D6,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.24.255.254")</f>
         <v>10.24.255.254</v>
       </c>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
+      <c r="I6" s="6">
+        <v>10</v>
+      </c>
+      <c r="J6" s="20">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
@@ -6028,8 +6178,12 @@
         <f ca="1">IFERROR(__xludf.DUMMYFUNCTION("REGEXREPLACE(D7,""\.[0-9]+\.[0-9]+$"","".255.254"")"),"10.34.255.254")</f>
         <v>10.34.255.254</v>
       </c>
-      <c r="I7" s="20"/>
-      <c r="J7" s="20"/>
+      <c r="I7" s="6">
+        <v>10</v>
+      </c>
+      <c r="J7" s="20">
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="22"/>

</xml_diff>

<commit_message>
added nat u testet
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nanik\Music\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC04455-DE09-4BB9-82E3-55A5CC03809B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D422DA-D1E2-4BF0-B67D-B73E42D50728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="52">
   <si>
     <t>site</t>
   </si>
@@ -186,6 +186,12 @@
   <si>
     <t>30.1-20.4</t>
   </si>
+  <si>
+    <t>isp_next_hop_addr</t>
+  </si>
+  <si>
+    <t>198.162.0.12</t>
+  </si>
 </sst>
 </file>
 
@@ -330,12 +336,30 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="138">
+  <dxfs count="139">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -497,6 +521,111 @@
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
@@ -566,111 +695,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -1313,100 +1337,100 @@
   </dxfs>
   <tableStyles count="16">
     <tableStyle name="Site 1 (HUB)-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="137"/>
-      <tableStyleElement type="headerRow" dxfId="136"/>
-      <tableStyleElement type="firstRowStripe" dxfId="135"/>
-      <tableStyleElement type="secondRowStripe" dxfId="134"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="138"/>
+      <tableStyleElement type="headerRow" dxfId="137"/>
+      <tableStyleElement type="firstRowStripe" dxfId="136"/>
+      <tableStyleElement type="secondRowStripe" dxfId="135"/>
     </tableStyle>
     <tableStyle name="Site 3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="133"/>
-      <tableStyleElement type="headerRow" dxfId="132"/>
-      <tableStyleElement type="firstRowStripe" dxfId="131"/>
-      <tableStyleElement type="secondRowStripe" dxfId="130"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="134"/>
+      <tableStyleElement type="headerRow" dxfId="133"/>
+      <tableStyleElement type="firstRowStripe" dxfId="132"/>
+      <tableStyleElement type="secondRowStripe" dxfId="131"/>
     </tableStyle>
     <tableStyle name="Site 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="129"/>
-      <tableStyleElement type="headerRow" dxfId="128"/>
-      <tableStyleElement type="firstRowStripe" dxfId="127"/>
-      <tableStyleElement type="secondRowStripe" dxfId="126"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="130"/>
+      <tableStyleElement type="headerRow" dxfId="129"/>
+      <tableStyleElement type="firstRowStripe" dxfId="128"/>
+      <tableStyleElement type="secondRowStripe" dxfId="127"/>
     </tableStyle>
     <tableStyle name="Site 4-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="125"/>
-      <tableStyleElement type="headerRow" dxfId="124"/>
-      <tableStyleElement type="firstRowStripe" dxfId="123"/>
-      <tableStyleElement type="secondRowStripe" dxfId="122"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="126"/>
+      <tableStyleElement type="headerRow" dxfId="125"/>
+      <tableStyleElement type="firstRowStripe" dxfId="124"/>
+      <tableStyleElement type="secondRowStripe" dxfId="123"/>
     </tableStyle>
     <tableStyle name="Site 3-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="121"/>
-      <tableStyleElement type="headerRow" dxfId="120"/>
-      <tableStyleElement type="firstRowStripe" dxfId="119"/>
-      <tableStyleElement type="secondRowStripe" dxfId="118"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="122"/>
+      <tableStyleElement type="headerRow" dxfId="121"/>
+      <tableStyleElement type="firstRowStripe" dxfId="120"/>
+      <tableStyleElement type="secondRowStripe" dxfId="119"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="117"/>
-      <tableStyleElement type="headerRow" dxfId="116"/>
-      <tableStyleElement type="firstRowStripe" dxfId="115"/>
-      <tableStyleElement type="secondRowStripe" dxfId="114"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="118"/>
+      <tableStyleElement type="headerRow" dxfId="117"/>
+      <tableStyleElement type="firstRowStripe" dxfId="116"/>
+      <tableStyleElement type="secondRowStripe" dxfId="115"/>
     </tableStyle>
     <tableStyle name="Site 2-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="113"/>
-      <tableStyleElement type="headerRow" dxfId="112"/>
-      <tableStyleElement type="firstRowStripe" dxfId="111"/>
-      <tableStyleElement type="secondRowStripe" dxfId="110"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="114"/>
+      <tableStyleElement type="headerRow" dxfId="113"/>
+      <tableStyleElement type="firstRowStripe" dxfId="112"/>
+      <tableStyleElement type="secondRowStripe" dxfId="111"/>
     </tableStyle>
     <tableStyle name="Site 3-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="109"/>
-      <tableStyleElement type="headerRow" dxfId="108"/>
-      <tableStyleElement type="firstRowStripe" dxfId="107"/>
-      <tableStyleElement type="secondRowStripe" dxfId="106"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="110"/>
+      <tableStyleElement type="headerRow" dxfId="109"/>
+      <tableStyleElement type="firstRowStripe" dxfId="108"/>
+      <tableStyleElement type="secondRowStripe" dxfId="107"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF08000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="105"/>
-      <tableStyleElement type="headerRow" dxfId="104"/>
-      <tableStyleElement type="firstRowStripe" dxfId="103"/>
-      <tableStyleElement type="secondRowStripe" dxfId="102"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="106"/>
+      <tableStyleElement type="headerRow" dxfId="105"/>
+      <tableStyleElement type="firstRowStripe" dxfId="104"/>
+      <tableStyleElement type="secondRowStripe" dxfId="103"/>
     </tableStyle>
     <tableStyle name="Site 4-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF09000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="101"/>
-      <tableStyleElement type="headerRow" dxfId="100"/>
-      <tableStyleElement type="firstRowStripe" dxfId="99"/>
-      <tableStyleElement type="secondRowStripe" dxfId="98"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="102"/>
+      <tableStyleElement type="headerRow" dxfId="101"/>
+      <tableStyleElement type="firstRowStripe" dxfId="100"/>
+      <tableStyleElement type="secondRowStripe" dxfId="99"/>
     </tableStyle>
     <tableStyle name="Site 3-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0A000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="97"/>
-      <tableStyleElement type="headerRow" dxfId="96"/>
-      <tableStyleElement type="firstRowStripe" dxfId="95"/>
-      <tableStyleElement type="secondRowStripe" dxfId="94"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="98"/>
+      <tableStyleElement type="headerRow" dxfId="97"/>
+      <tableStyleElement type="firstRowStripe" dxfId="96"/>
+      <tableStyleElement type="secondRowStripe" dxfId="95"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0B000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="93"/>
-      <tableStyleElement type="headerRow" dxfId="92"/>
-      <tableStyleElement type="firstRowStripe" dxfId="91"/>
-      <tableStyleElement type="secondRowStripe" dxfId="90"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="94"/>
+      <tableStyleElement type="headerRow" dxfId="93"/>
+      <tableStyleElement type="firstRowStripe" dxfId="92"/>
+      <tableStyleElement type="secondRowStripe" dxfId="91"/>
     </tableStyle>
     <tableStyle name="Site 2-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0C000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="89"/>
-      <tableStyleElement type="headerRow" dxfId="88"/>
-      <tableStyleElement type="firstRowStripe" dxfId="87"/>
-      <tableStyleElement type="secondRowStripe" dxfId="86"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="90"/>
+      <tableStyleElement type="headerRow" dxfId="89"/>
+      <tableStyleElement type="firstRowStripe" dxfId="88"/>
+      <tableStyleElement type="secondRowStripe" dxfId="87"/>
     </tableStyle>
     <tableStyle name="Site 4-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0D000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="85"/>
-      <tableStyleElement type="headerRow" dxfId="84"/>
-      <tableStyleElement type="firstRowStripe" dxfId="83"/>
-      <tableStyleElement type="secondRowStripe" dxfId="82"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="86"/>
+      <tableStyleElement type="headerRow" dxfId="85"/>
+      <tableStyleElement type="firstRowStripe" dxfId="84"/>
+      <tableStyleElement type="secondRowStripe" dxfId="83"/>
     </tableStyle>
     <tableStyle name="Site 2-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0E000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="81"/>
-      <tableStyleElement type="headerRow" dxfId="80"/>
-      <tableStyleElement type="firstRowStripe" dxfId="79"/>
-      <tableStyleElement type="secondRowStripe" dxfId="78"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="82"/>
+      <tableStyleElement type="headerRow" dxfId="81"/>
+      <tableStyleElement type="firstRowStripe" dxfId="80"/>
+      <tableStyleElement type="secondRowStripe" dxfId="79"/>
     </tableStyle>
     <tableStyle name="Site 4-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0F000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="77"/>
-      <tableStyleElement type="headerRow" dxfId="76"/>
-      <tableStyleElement type="firstRowStripe" dxfId="75"/>
-      <tableStyleElement type="secondRowStripe" dxfId="74"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="78"/>
+      <tableStyleElement type="headerRow" dxfId="77"/>
+      <tableStyleElement type="firstRowStripe" dxfId="76"/>
+      <tableStyleElement type="secondRowStripe" dxfId="75"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1421,14 +1445,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:F2">
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:G2">
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="site"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="intf_prefix"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="router-id"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
+    <tableColumn id="7" xr3:uid="{317330A8-84F0-4160-B3DB-F31DCF020098}" name="isp_next_hop_addr" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Site 1 (HUB)-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1453,37 +1478,37 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="72" dataDxfId="71" totalsRowDxfId="70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="49" dataDxfId="48" totalsRowDxfId="47">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="69">
+    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="46">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="68"/>
-    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="66" totalsRowDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="43" totalsRowDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{0D1C10A1-9717-4057-887E-5357402CB0E7}" name="Tabell1618242833" displayName="Tabell1618242833" ref="A21:I23" headerRowDxfId="64" dataDxfId="63" totalsRowDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{0D1C10A1-9717-4057-887E-5357402CB0E7}" name="Tabell1618242833" displayName="Tabell1618242833" ref="A21:I23" headerRowDxfId="41" dataDxfId="40" totalsRowDxfId="39">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{85F36277-7C1F-4D2C-A112-F88A589A07DE}" name="SW" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{5147590E-0FE4-463A-9241-58FBD204D8DE}" name="MGMT Vlan" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{F8B990D7-C517-482F-BAFB-8EA413932149}" name="MGMT ip" dataDxfId="59">
+    <tableColumn id="1" xr3:uid="{85F36277-7C1F-4D2C-A112-F88A589A07DE}" name="SW" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{5147590E-0FE4-463A-9241-58FBD204D8DE}" name="MGMT Vlan" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{F8B990D7-C517-482F-BAFB-8EA413932149}" name="MGMT ip" dataDxfId="36">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BCAF6C67-3F43-4FFA-8105-4158589FBEBF}" name="gateway" dataDxfId="58">
+    <tableColumn id="4" xr3:uid="{BCAF6C67-3F43-4FFA-8105-4158589FBEBF}" name="gateway" dataDxfId="35">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D20CE737-A3E7-4538-BC2C-E8176E6D9EE6}" name="mask" dataDxfId="57">
+    <tableColumn id="5" xr3:uid="{D20CE737-A3E7-4538-BC2C-E8176E6D9EE6}" name="mask" dataDxfId="34">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9365541B-740A-44C6-ADF0-F56C3A9D13D1}" name="vlan-antall" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{7551B7F0-84D1-4CCD-9D8E-AEF551C0B4CA}" name="num_ports" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{7717CEDF-A842-4402-B477-8AD92D9C9A65}" name="intf_prefix" dataDxfId="52" totalsRowDxfId="51"/>
-    <tableColumn id="9" xr3:uid="{31DB8A8F-54E2-45C5-B25D-6C92CA4826D3}" name="num_port_ledig" dataDxfId="50" totalsRowDxfId="49">
+    <tableColumn id="6" xr3:uid="{9365541B-740A-44C6-ADF0-F56C3A9D13D1}" name="vlan-antall" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{7551B7F0-84D1-4CCD-9D8E-AEF551C0B4CA}" name="num_ports" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{7717CEDF-A842-4402-B477-8AD92D9C9A65}" name="intf_prefix" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{31DB8A8F-54E2-45C5-B25D-6C92CA4826D3}" name="num_port_ledig" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1522,7 +1547,7 @@
       <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{90B6F7A5-9BD7-49C1-B978-43855C69778B}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{924908E3-556A-40DC-9275-15A17DCB79EE}" name="antall-res" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{924908E3-556A-40DC-9275-15A17DCB79EE}" name="antall-res" dataDxfId="25"/>
     <tableColumn id="10" xr3:uid="{06C63977-B34D-4B5A-A3DF-C4469BD779D7}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{3BCA4967-58B4-4E19-8D6C-1D7A65EE09F2}" name="pri-1-10"/>
   </tableColumns>
@@ -1563,37 +1588,37 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{BF23752F-BD82-401A-981D-B03F45E60744}" name="Tabell1319253010" displayName="Tabell1319253010" ref="A18:D19" headerRowDxfId="23" dataDxfId="22" totalsRowDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{BF23752F-BD82-401A-981D-B03F45E60744}" name="Tabell1319253010" displayName="Tabell1319253010" ref="A18:D19" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C10764F4-CFFC-4EE6-9EEA-82891DC993E3}" name="site" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{C10764F4-CFFC-4EE6-9EEA-82891DC993E3}" name="site" dataDxfId="21">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{495F2DCB-B8C1-4ED6-89E5-8F715B0716BB}" name="brukernavn" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{0AF6FD65-2F7E-47E7-AC42-98BED9837A14}" name="passord" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{817B17C3-5974-47D5-8903-3EB5C370F4C0}" name="vty_lines" dataDxfId="16" totalsRowDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{495F2DCB-B8C1-4ED6-89E5-8F715B0716BB}" name="brukernavn" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{0AF6FD65-2F7E-47E7-AC42-98BED9837A14}" name="passord" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{817B17C3-5974-47D5-8903-3EB5C370F4C0}" name="vty_lines" dataDxfId="18" totalsRowDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{131BE48E-0BD4-4282-9346-3A5772CD50CB}" name="Tabell161824283312" displayName="Tabell161824283312" ref="A21:I23" headerRowDxfId="15" dataDxfId="14" totalsRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{131BE48E-0BD4-4282-9346-3A5772CD50CB}" name="Tabell161824283312" displayName="Tabell161824283312" ref="A21:I23" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{72296002-AE4E-4E82-8305-4DDD12CA9BE2}" name="SW" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{2973A27B-3C31-4DE1-A0D7-9AC4974D229E}" name="MGMT Vlan" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{FBB420D8-ADD0-4632-A43B-10F32DF3105D}" name="MGMT ip" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{72296002-AE4E-4E82-8305-4DDD12CA9BE2}" name="SW" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{2973A27B-3C31-4DE1-A0D7-9AC4974D229E}" name="MGMT Vlan" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{FBB420D8-ADD0-4632-A43B-10F32DF3105D}" name="MGMT ip" dataDxfId="11">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7D99B76D-9B56-49C4-9B59-4DED1EAF6B17}" name="gateway" dataDxfId="9">
+    <tableColumn id="4" xr3:uid="{7D99B76D-9B56-49C4-9B59-4DED1EAF6B17}" name="gateway" dataDxfId="10">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{E0CF3890-FEBD-4B81-ABF6-157ECCA5F3A4}" name="mask" dataDxfId="8">
+    <tableColumn id="5" xr3:uid="{E0CF3890-FEBD-4B81-ABF6-157ECCA5F3A4}" name="mask" dataDxfId="9">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4941A454-E75E-46D9-BD24-7C44A665D3F6}" name="vlan-antall" dataDxfId="6" totalsRowDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{08C93E9C-BB70-4A35-9AFF-1C123A3CD9A9}" name="num_ports" dataDxfId="4" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{4BBEDCD8-9032-4F13-A138-6E836EDDF4D2}" name="intf_prefix" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{2E94FBF2-04F2-4961-A5CD-DC3BCD091189}" name="num_port_ledig" dataDxfId="0" totalsRowDxfId="1">
+    <tableColumn id="6" xr3:uid="{4941A454-E75E-46D9-BD24-7C44A665D3F6}" name="vlan-antall" dataDxfId="8" totalsRowDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{08C93E9C-BB70-4A35-9AFF-1C123A3CD9A9}" name="num_ports" dataDxfId="6" totalsRowDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{4BBEDCD8-9032-4F13-A138-6E836EDDF4D2}" name="intf_prefix" dataDxfId="4" totalsRowDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{2E94FBF2-04F2-4961-A5CD-DC3BCD091189}" name="num_port_ledig" dataDxfId="2" totalsRowDxfId="1">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1612,7 +1637,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="74"/>
     <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{BBB41126-CDAD-40BD-92C3-0A8EEC64127E}" name="pri-1-10"/>
   </tableColumns>
@@ -1651,37 +1676,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="47" dataDxfId="46" totalsRowDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="73" dataDxfId="72" totalsRowDxfId="71">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="44">
+    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="70">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="67"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" headerRowDxfId="40" dataDxfId="39" totalsRowDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" headerRowDxfId="66" dataDxfId="65" totalsRowDxfId="64">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="35">
+    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="61">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="34">
+    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="60">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="33">
+    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="59">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="32" totalsRowDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="30" totalsRowDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="26" totalsRowDxfId="25">
+    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="58" totalsRowDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="52" totalsRowDxfId="51">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1714,7 +1739,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="50"/>
     <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{1CC9D42E-8B8D-4781-B4E6-7B024D0D4DB5}" name="pri-1-10"/>
   </tableColumns>
@@ -1942,6 +1967,7 @@
     <col min="2" max="2" width="12.6640625" customWidth="1"/>
     <col min="3" max="4" width="23.88671875" customWidth="1"/>
     <col min="5" max="6" width="12.5546875" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" customWidth="1"/>
     <col min="9" max="9" width="18.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1964,6 +1990,9 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -1984,6 +2013,9 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5358,7 +5390,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
bedre strat for å hente isp gatway
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nanik\Music\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D422DA-D1E2-4BF0-B67D-B73E42D50728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76F3C545-E422-41E8-BD17-30F4FBE8979C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="50">
   <si>
     <t>site</t>
   </si>
@@ -186,12 +186,6 @@
   <si>
     <t>30.1-20.4</t>
   </si>
-  <si>
-    <t>isp_next_hop_addr</t>
-  </si>
-  <si>
-    <t>198.162.0.12</t>
-  </si>
 </sst>
 </file>
 
@@ -336,25 +330,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="139">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="138">
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1337,100 +1313,100 @@
   </dxfs>
   <tableStyles count="16">
     <tableStyle name="Site 1 (HUB)-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="138"/>
-      <tableStyleElement type="headerRow" dxfId="137"/>
-      <tableStyleElement type="firstRowStripe" dxfId="136"/>
-      <tableStyleElement type="secondRowStripe" dxfId="135"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="137"/>
+      <tableStyleElement type="headerRow" dxfId="136"/>
+      <tableStyleElement type="firstRowStripe" dxfId="135"/>
+      <tableStyleElement type="secondRowStripe" dxfId="134"/>
     </tableStyle>
     <tableStyle name="Site 3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="134"/>
-      <tableStyleElement type="headerRow" dxfId="133"/>
-      <tableStyleElement type="firstRowStripe" dxfId="132"/>
-      <tableStyleElement type="secondRowStripe" dxfId="131"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="133"/>
+      <tableStyleElement type="headerRow" dxfId="132"/>
+      <tableStyleElement type="firstRowStripe" dxfId="131"/>
+      <tableStyleElement type="secondRowStripe" dxfId="130"/>
     </tableStyle>
     <tableStyle name="Site 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="130"/>
-      <tableStyleElement type="headerRow" dxfId="129"/>
-      <tableStyleElement type="firstRowStripe" dxfId="128"/>
-      <tableStyleElement type="secondRowStripe" dxfId="127"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="129"/>
+      <tableStyleElement type="headerRow" dxfId="128"/>
+      <tableStyleElement type="firstRowStripe" dxfId="127"/>
+      <tableStyleElement type="secondRowStripe" dxfId="126"/>
     </tableStyle>
     <tableStyle name="Site 4-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="126"/>
-      <tableStyleElement type="headerRow" dxfId="125"/>
-      <tableStyleElement type="firstRowStripe" dxfId="124"/>
-      <tableStyleElement type="secondRowStripe" dxfId="123"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="125"/>
+      <tableStyleElement type="headerRow" dxfId="124"/>
+      <tableStyleElement type="firstRowStripe" dxfId="123"/>
+      <tableStyleElement type="secondRowStripe" dxfId="122"/>
     </tableStyle>
     <tableStyle name="Site 3-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="122"/>
-      <tableStyleElement type="headerRow" dxfId="121"/>
-      <tableStyleElement type="firstRowStripe" dxfId="120"/>
-      <tableStyleElement type="secondRowStripe" dxfId="119"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="121"/>
+      <tableStyleElement type="headerRow" dxfId="120"/>
+      <tableStyleElement type="firstRowStripe" dxfId="119"/>
+      <tableStyleElement type="secondRowStripe" dxfId="118"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="118"/>
-      <tableStyleElement type="headerRow" dxfId="117"/>
-      <tableStyleElement type="firstRowStripe" dxfId="116"/>
-      <tableStyleElement type="secondRowStripe" dxfId="115"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="117"/>
+      <tableStyleElement type="headerRow" dxfId="116"/>
+      <tableStyleElement type="firstRowStripe" dxfId="115"/>
+      <tableStyleElement type="secondRowStripe" dxfId="114"/>
     </tableStyle>
     <tableStyle name="Site 2-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="114"/>
-      <tableStyleElement type="headerRow" dxfId="113"/>
-      <tableStyleElement type="firstRowStripe" dxfId="112"/>
-      <tableStyleElement type="secondRowStripe" dxfId="111"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="113"/>
+      <tableStyleElement type="headerRow" dxfId="112"/>
+      <tableStyleElement type="firstRowStripe" dxfId="111"/>
+      <tableStyleElement type="secondRowStripe" dxfId="110"/>
     </tableStyle>
     <tableStyle name="Site 3-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="110"/>
-      <tableStyleElement type="headerRow" dxfId="109"/>
-      <tableStyleElement type="firstRowStripe" dxfId="108"/>
-      <tableStyleElement type="secondRowStripe" dxfId="107"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="109"/>
+      <tableStyleElement type="headerRow" dxfId="108"/>
+      <tableStyleElement type="firstRowStripe" dxfId="107"/>
+      <tableStyleElement type="secondRowStripe" dxfId="106"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF08000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="106"/>
-      <tableStyleElement type="headerRow" dxfId="105"/>
-      <tableStyleElement type="firstRowStripe" dxfId="104"/>
-      <tableStyleElement type="secondRowStripe" dxfId="103"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="105"/>
+      <tableStyleElement type="headerRow" dxfId="104"/>
+      <tableStyleElement type="firstRowStripe" dxfId="103"/>
+      <tableStyleElement type="secondRowStripe" dxfId="102"/>
     </tableStyle>
     <tableStyle name="Site 4-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF09000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="102"/>
-      <tableStyleElement type="headerRow" dxfId="101"/>
-      <tableStyleElement type="firstRowStripe" dxfId="100"/>
-      <tableStyleElement type="secondRowStripe" dxfId="99"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="101"/>
+      <tableStyleElement type="headerRow" dxfId="100"/>
+      <tableStyleElement type="firstRowStripe" dxfId="99"/>
+      <tableStyleElement type="secondRowStripe" dxfId="98"/>
     </tableStyle>
     <tableStyle name="Site 3-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0A000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="98"/>
-      <tableStyleElement type="headerRow" dxfId="97"/>
-      <tableStyleElement type="firstRowStripe" dxfId="96"/>
-      <tableStyleElement type="secondRowStripe" dxfId="95"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="97"/>
+      <tableStyleElement type="headerRow" dxfId="96"/>
+      <tableStyleElement type="firstRowStripe" dxfId="95"/>
+      <tableStyleElement type="secondRowStripe" dxfId="94"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0B000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="94"/>
-      <tableStyleElement type="headerRow" dxfId="93"/>
-      <tableStyleElement type="firstRowStripe" dxfId="92"/>
-      <tableStyleElement type="secondRowStripe" dxfId="91"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="93"/>
+      <tableStyleElement type="headerRow" dxfId="92"/>
+      <tableStyleElement type="firstRowStripe" dxfId="91"/>
+      <tableStyleElement type="secondRowStripe" dxfId="90"/>
     </tableStyle>
     <tableStyle name="Site 2-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0C000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="90"/>
-      <tableStyleElement type="headerRow" dxfId="89"/>
-      <tableStyleElement type="firstRowStripe" dxfId="88"/>
-      <tableStyleElement type="secondRowStripe" dxfId="87"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="89"/>
+      <tableStyleElement type="headerRow" dxfId="88"/>
+      <tableStyleElement type="firstRowStripe" dxfId="87"/>
+      <tableStyleElement type="secondRowStripe" dxfId="86"/>
     </tableStyle>
     <tableStyle name="Site 4-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0D000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="86"/>
-      <tableStyleElement type="headerRow" dxfId="85"/>
-      <tableStyleElement type="firstRowStripe" dxfId="84"/>
-      <tableStyleElement type="secondRowStripe" dxfId="83"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="85"/>
+      <tableStyleElement type="headerRow" dxfId="84"/>
+      <tableStyleElement type="firstRowStripe" dxfId="83"/>
+      <tableStyleElement type="secondRowStripe" dxfId="82"/>
     </tableStyle>
     <tableStyle name="Site 2-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0E000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="82"/>
-      <tableStyleElement type="headerRow" dxfId="81"/>
-      <tableStyleElement type="firstRowStripe" dxfId="80"/>
-      <tableStyleElement type="secondRowStripe" dxfId="79"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="81"/>
+      <tableStyleElement type="headerRow" dxfId="80"/>
+      <tableStyleElement type="firstRowStripe" dxfId="79"/>
+      <tableStyleElement type="secondRowStripe" dxfId="78"/>
     </tableStyle>
     <tableStyle name="Site 4-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0F000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="78"/>
-      <tableStyleElement type="headerRow" dxfId="77"/>
-      <tableStyleElement type="firstRowStripe" dxfId="76"/>
-      <tableStyleElement type="secondRowStripe" dxfId="75"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="77"/>
+      <tableStyleElement type="headerRow" dxfId="76"/>
+      <tableStyleElement type="firstRowStripe" dxfId="75"/>
+      <tableStyleElement type="secondRowStripe" dxfId="74"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1445,15 +1421,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:G2">
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:F2">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="site"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="intf_prefix"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="router-id"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
-    <tableColumn id="7" xr3:uid="{317330A8-84F0-4160-B3DB-F31DCF020098}" name="isp_next_hop_addr" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Site 1 (HUB)-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1478,37 +1453,37 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="49" dataDxfId="48" totalsRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="48" dataDxfId="47" totalsRowDxfId="46">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="46">
+    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="45">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="42" totalsRowDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{0D1C10A1-9717-4057-887E-5357402CB0E7}" name="Tabell1618242833" displayName="Tabell1618242833" ref="A21:I23" headerRowDxfId="41" dataDxfId="40" totalsRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{0D1C10A1-9717-4057-887E-5357402CB0E7}" name="Tabell1618242833" displayName="Tabell1618242833" ref="A21:I23" headerRowDxfId="40" dataDxfId="39" totalsRowDxfId="38">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{85F36277-7C1F-4D2C-A112-F88A589A07DE}" name="SW" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{5147590E-0FE4-463A-9241-58FBD204D8DE}" name="MGMT Vlan" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{F8B990D7-C517-482F-BAFB-8EA413932149}" name="MGMT ip" dataDxfId="36">
+    <tableColumn id="1" xr3:uid="{85F36277-7C1F-4D2C-A112-F88A589A07DE}" name="SW" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{5147590E-0FE4-463A-9241-58FBD204D8DE}" name="MGMT Vlan" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{F8B990D7-C517-482F-BAFB-8EA413932149}" name="MGMT ip" dataDxfId="35">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BCAF6C67-3F43-4FFA-8105-4158589FBEBF}" name="gateway" dataDxfId="35">
+    <tableColumn id="4" xr3:uid="{BCAF6C67-3F43-4FFA-8105-4158589FBEBF}" name="gateway" dataDxfId="34">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D20CE737-A3E7-4538-BC2C-E8176E6D9EE6}" name="mask" dataDxfId="34">
+    <tableColumn id="5" xr3:uid="{D20CE737-A3E7-4538-BC2C-E8176E6D9EE6}" name="mask" dataDxfId="33">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{9365541B-740A-44C6-ADF0-F56C3A9D13D1}" name="vlan-antall" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{7551B7F0-84D1-4CCD-9D8E-AEF551C0B4CA}" name="num_ports" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{7717CEDF-A842-4402-B477-8AD92D9C9A65}" name="intf_prefix" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{31DB8A8F-54E2-45C5-B25D-6C92CA4826D3}" name="num_port_ledig" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="6" xr3:uid="{9365541B-740A-44C6-ADF0-F56C3A9D13D1}" name="vlan-antall" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{7551B7F0-84D1-4CCD-9D8E-AEF551C0B4CA}" name="num_ports" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{7717CEDF-A842-4402-B477-8AD92D9C9A65}" name="intf_prefix" dataDxfId="28" totalsRowDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{31DB8A8F-54E2-45C5-B25D-6C92CA4826D3}" name="num_port_ledig" dataDxfId="26" totalsRowDxfId="25">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1547,7 +1522,7 @@
       <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{90B6F7A5-9BD7-49C1-B978-43855C69778B}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{924908E3-556A-40DC-9275-15A17DCB79EE}" name="antall-res" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{924908E3-556A-40DC-9275-15A17DCB79EE}" name="antall-res" dataDxfId="24"/>
     <tableColumn id="10" xr3:uid="{06C63977-B34D-4B5A-A3DF-C4469BD779D7}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{3BCA4967-58B4-4E19-8D6C-1D7A65EE09F2}" name="pri-1-10"/>
   </tableColumns>
@@ -1588,37 +1563,37 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{BF23752F-BD82-401A-981D-B03F45E60744}" name="Tabell1319253010" displayName="Tabell1319253010" ref="A18:D19" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{BF23752F-BD82-401A-981D-B03F45E60744}" name="Tabell1319253010" displayName="Tabell1319253010" ref="A18:D19" headerRowDxfId="23" dataDxfId="22" totalsRowDxfId="21">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C10764F4-CFFC-4EE6-9EEA-82891DC993E3}" name="site" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{C10764F4-CFFC-4EE6-9EEA-82891DC993E3}" name="site" dataDxfId="20">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{495F2DCB-B8C1-4ED6-89E5-8F715B0716BB}" name="brukernavn" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{0AF6FD65-2F7E-47E7-AC42-98BED9837A14}" name="passord" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{817B17C3-5974-47D5-8903-3EB5C370F4C0}" name="vty_lines" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{495F2DCB-B8C1-4ED6-89E5-8F715B0716BB}" name="brukernavn" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{0AF6FD65-2F7E-47E7-AC42-98BED9837A14}" name="passord" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{817B17C3-5974-47D5-8903-3EB5C370F4C0}" name="vty_lines" dataDxfId="17" totalsRowDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{131BE48E-0BD4-4282-9346-3A5772CD50CB}" name="Tabell161824283312" displayName="Tabell161824283312" ref="A21:I23" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{131BE48E-0BD4-4282-9346-3A5772CD50CB}" name="Tabell161824283312" displayName="Tabell161824283312" ref="A21:I23" headerRowDxfId="15" dataDxfId="14" totalsRowDxfId="13">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{72296002-AE4E-4E82-8305-4DDD12CA9BE2}" name="SW" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{2973A27B-3C31-4DE1-A0D7-9AC4974D229E}" name="MGMT Vlan" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{FBB420D8-ADD0-4632-A43B-10F32DF3105D}" name="MGMT ip" dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{72296002-AE4E-4E82-8305-4DDD12CA9BE2}" name="SW" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{2973A27B-3C31-4DE1-A0D7-9AC4974D229E}" name="MGMT Vlan" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{FBB420D8-ADD0-4632-A43B-10F32DF3105D}" name="MGMT ip" dataDxfId="10">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{7D99B76D-9B56-49C4-9B59-4DED1EAF6B17}" name="gateway" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{7D99B76D-9B56-49C4-9B59-4DED1EAF6B17}" name="gateway" dataDxfId="9">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{E0CF3890-FEBD-4B81-ABF6-157ECCA5F3A4}" name="mask" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{E0CF3890-FEBD-4B81-ABF6-157ECCA5F3A4}" name="mask" dataDxfId="8">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{4941A454-E75E-46D9-BD24-7C44A665D3F6}" name="vlan-antall" dataDxfId="8" totalsRowDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{08C93E9C-BB70-4A35-9AFF-1C123A3CD9A9}" name="num_ports" dataDxfId="6" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{4BBEDCD8-9032-4F13-A138-6E836EDDF4D2}" name="intf_prefix" dataDxfId="4" totalsRowDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{2E94FBF2-04F2-4961-A5CD-DC3BCD091189}" name="num_port_ledig" dataDxfId="2" totalsRowDxfId="1">
+    <tableColumn id="6" xr3:uid="{4941A454-E75E-46D9-BD24-7C44A665D3F6}" name="vlan-antall" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{08C93E9C-BB70-4A35-9AFF-1C123A3CD9A9}" name="num_ports" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{4BBEDCD8-9032-4F13-A138-6E836EDDF4D2}" name="intf_prefix" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{2E94FBF2-04F2-4961-A5CD-DC3BCD091189}" name="num_port_ledig" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1637,7 +1612,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="74"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="73"/>
     <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{BBB41126-CDAD-40BD-92C3-0A8EEC64127E}" name="pri-1-10"/>
   </tableColumns>
@@ -1676,37 +1651,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="73" dataDxfId="72" totalsRowDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="72" dataDxfId="71" totalsRowDxfId="70">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="70">
+    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="69">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="69"/>
-    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="68"/>
-    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" headerRowDxfId="66" dataDxfId="65" totalsRowDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" headerRowDxfId="65" dataDxfId="64" totalsRowDxfId="63">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="61">
+    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="60">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="60">
+    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="59">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="59">
+    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="58">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="58" totalsRowDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="52" totalsRowDxfId="51">
+    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="57" totalsRowDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="55" totalsRowDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="51" totalsRowDxfId="50">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1739,7 +1714,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="49"/>
     <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{1CC9D42E-8B8D-4781-B4E6-7B024D0D4DB5}" name="pri-1-10"/>
   </tableColumns>
@@ -1990,9 +1965,6 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -2013,9 +1985,6 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
navn fiks litt penerer
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4FB680-C061-4FAC-AA77-E5AEE21A30C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575F4A5D-A441-4C0F-800A-E462E8EED511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="51">
   <si>
     <t>site</t>
   </si>
@@ -181,6 +181,12 @@
   </si>
   <si>
     <t>pri-afxx</t>
+  </si>
+  <si>
+    <t>30.2-20.5</t>
+  </si>
+  <si>
+    <t>20.1-10.1</t>
   </si>
 </sst>
 </file>
@@ -276,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -319,35 +325,41 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="113">
-    <dxf>
+  <dxfs count="111">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -363,14 +375,83 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
         <sz val="11"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -442,49 +523,10 @@
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1201,100 +1243,100 @@
   </dxfs>
   <tableStyles count="16">
     <tableStyle name="Site 1 (HUB)-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="112"/>
-      <tableStyleElement type="headerRow" dxfId="111"/>
-      <tableStyleElement type="firstRowStripe" dxfId="110"/>
-      <tableStyleElement type="secondRowStripe" dxfId="109"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="110"/>
+      <tableStyleElement type="headerRow" dxfId="109"/>
+      <tableStyleElement type="firstRowStripe" dxfId="108"/>
+      <tableStyleElement type="secondRowStripe" dxfId="107"/>
     </tableStyle>
     <tableStyle name="Site 3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="108"/>
-      <tableStyleElement type="headerRow" dxfId="107"/>
-      <tableStyleElement type="firstRowStripe" dxfId="106"/>
-      <tableStyleElement type="secondRowStripe" dxfId="105"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="106"/>
+      <tableStyleElement type="headerRow" dxfId="105"/>
+      <tableStyleElement type="firstRowStripe" dxfId="104"/>
+      <tableStyleElement type="secondRowStripe" dxfId="103"/>
     </tableStyle>
     <tableStyle name="Site 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="104"/>
-      <tableStyleElement type="headerRow" dxfId="103"/>
-      <tableStyleElement type="firstRowStripe" dxfId="102"/>
-      <tableStyleElement type="secondRowStripe" dxfId="101"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="102"/>
+      <tableStyleElement type="headerRow" dxfId="101"/>
+      <tableStyleElement type="firstRowStripe" dxfId="100"/>
+      <tableStyleElement type="secondRowStripe" dxfId="99"/>
     </tableStyle>
     <tableStyle name="Site 4-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="100"/>
-      <tableStyleElement type="headerRow" dxfId="99"/>
-      <tableStyleElement type="firstRowStripe" dxfId="98"/>
-      <tableStyleElement type="secondRowStripe" dxfId="97"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="98"/>
+      <tableStyleElement type="headerRow" dxfId="97"/>
+      <tableStyleElement type="firstRowStripe" dxfId="96"/>
+      <tableStyleElement type="secondRowStripe" dxfId="95"/>
     </tableStyle>
     <tableStyle name="Site 3-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="96"/>
-      <tableStyleElement type="headerRow" dxfId="95"/>
-      <tableStyleElement type="firstRowStripe" dxfId="94"/>
-      <tableStyleElement type="secondRowStripe" dxfId="93"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="94"/>
+      <tableStyleElement type="headerRow" dxfId="93"/>
+      <tableStyleElement type="firstRowStripe" dxfId="92"/>
+      <tableStyleElement type="secondRowStripe" dxfId="91"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="92"/>
-      <tableStyleElement type="headerRow" dxfId="91"/>
-      <tableStyleElement type="firstRowStripe" dxfId="90"/>
-      <tableStyleElement type="secondRowStripe" dxfId="89"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="90"/>
+      <tableStyleElement type="headerRow" dxfId="89"/>
+      <tableStyleElement type="firstRowStripe" dxfId="88"/>
+      <tableStyleElement type="secondRowStripe" dxfId="87"/>
     </tableStyle>
     <tableStyle name="Site 2-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="88"/>
-      <tableStyleElement type="headerRow" dxfId="87"/>
-      <tableStyleElement type="firstRowStripe" dxfId="86"/>
-      <tableStyleElement type="secondRowStripe" dxfId="85"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="86"/>
+      <tableStyleElement type="headerRow" dxfId="85"/>
+      <tableStyleElement type="firstRowStripe" dxfId="84"/>
+      <tableStyleElement type="secondRowStripe" dxfId="83"/>
     </tableStyle>
     <tableStyle name="Site 3-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="84"/>
-      <tableStyleElement type="headerRow" dxfId="83"/>
-      <tableStyleElement type="firstRowStripe" dxfId="82"/>
-      <tableStyleElement type="secondRowStripe" dxfId="81"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="82"/>
+      <tableStyleElement type="headerRow" dxfId="81"/>
+      <tableStyleElement type="firstRowStripe" dxfId="80"/>
+      <tableStyleElement type="secondRowStripe" dxfId="79"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF08000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="80"/>
-      <tableStyleElement type="headerRow" dxfId="79"/>
-      <tableStyleElement type="firstRowStripe" dxfId="78"/>
-      <tableStyleElement type="secondRowStripe" dxfId="77"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="78"/>
+      <tableStyleElement type="headerRow" dxfId="77"/>
+      <tableStyleElement type="firstRowStripe" dxfId="76"/>
+      <tableStyleElement type="secondRowStripe" dxfId="75"/>
     </tableStyle>
     <tableStyle name="Site 4-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF09000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="76"/>
-      <tableStyleElement type="headerRow" dxfId="75"/>
-      <tableStyleElement type="firstRowStripe" dxfId="74"/>
-      <tableStyleElement type="secondRowStripe" dxfId="73"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="74"/>
+      <tableStyleElement type="headerRow" dxfId="73"/>
+      <tableStyleElement type="firstRowStripe" dxfId="72"/>
+      <tableStyleElement type="secondRowStripe" dxfId="71"/>
     </tableStyle>
     <tableStyle name="Site 3-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0A000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="72"/>
-      <tableStyleElement type="headerRow" dxfId="71"/>
-      <tableStyleElement type="firstRowStripe" dxfId="70"/>
-      <tableStyleElement type="secondRowStripe" dxfId="69"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="70"/>
+      <tableStyleElement type="headerRow" dxfId="69"/>
+      <tableStyleElement type="firstRowStripe" dxfId="68"/>
+      <tableStyleElement type="secondRowStripe" dxfId="67"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0B000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="68"/>
-      <tableStyleElement type="headerRow" dxfId="67"/>
-      <tableStyleElement type="firstRowStripe" dxfId="66"/>
-      <tableStyleElement type="secondRowStripe" dxfId="65"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="66"/>
+      <tableStyleElement type="headerRow" dxfId="65"/>
+      <tableStyleElement type="firstRowStripe" dxfId="64"/>
+      <tableStyleElement type="secondRowStripe" dxfId="63"/>
     </tableStyle>
     <tableStyle name="Site 2-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0C000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="64"/>
-      <tableStyleElement type="headerRow" dxfId="63"/>
-      <tableStyleElement type="firstRowStripe" dxfId="62"/>
-      <tableStyleElement type="secondRowStripe" dxfId="61"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="62"/>
+      <tableStyleElement type="headerRow" dxfId="61"/>
+      <tableStyleElement type="firstRowStripe" dxfId="60"/>
+      <tableStyleElement type="secondRowStripe" dxfId="59"/>
     </tableStyle>
     <tableStyle name="Site 4-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0D000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="60"/>
-      <tableStyleElement type="headerRow" dxfId="59"/>
-      <tableStyleElement type="firstRowStripe" dxfId="58"/>
-      <tableStyleElement type="secondRowStripe" dxfId="57"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="58"/>
+      <tableStyleElement type="headerRow" dxfId="57"/>
+      <tableStyleElement type="firstRowStripe" dxfId="56"/>
+      <tableStyleElement type="secondRowStripe" dxfId="55"/>
     </tableStyle>
     <tableStyle name="Site 2-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0E000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="56"/>
-      <tableStyleElement type="headerRow" dxfId="55"/>
-      <tableStyleElement type="firstRowStripe" dxfId="54"/>
-      <tableStyleElement type="secondRowStripe" dxfId="53"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="54"/>
+      <tableStyleElement type="headerRow" dxfId="53"/>
+      <tableStyleElement type="firstRowStripe" dxfId="52"/>
+      <tableStyleElement type="secondRowStripe" dxfId="51"/>
     </tableStyle>
     <tableStyle name="Site 4-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0F000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="52"/>
-      <tableStyleElement type="headerRow" dxfId="51"/>
-      <tableStyleElement type="firstRowStripe" dxfId="50"/>
-      <tableStyleElement type="secondRowStripe" dxfId="49"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="50"/>
+      <tableStyleElement type="headerRow" dxfId="49"/>
+      <tableStyleElement type="firstRowStripe" dxfId="48"/>
+      <tableStyleElement type="secondRowStripe" dxfId="47"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1341,37 +1383,39 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="26" dataDxfId="25" totalsRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="33" dataDxfId="32" totalsRowDxfId="31">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="23">
+    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="30">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="20" totalsRowDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="27" totalsRowDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I22" headerRowDxfId="15" dataDxfId="14" totalsRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I24" headerRowDxfId="23" totalsRowDxfId="22">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="8">
+      <calculatedColumnFormula>ROW()-21</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="6">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="9">
+    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="5">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="8">
+    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="4">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="6" totalsRowDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="4" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="2" totalsRowDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="0" totalsRowDxfId="1">
+    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="3" totalsRowDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="2" totalsRowDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="1" totalsRowDxfId="19"/>
+    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="0" totalsRowDxfId="18">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1390,7 +1434,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="48"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="46"/>
     <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{BBB41126-CDAD-40BD-92C3-0A8EEC64127E}" name="pri-1-10"/>
   </tableColumns>
@@ -1429,37 +1473,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="47" dataDxfId="46" totalsRowDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="45" dataDxfId="44" totalsRowDxfId="43">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="44">
+    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="42">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" insertRow="1" headerRowDxfId="18" dataDxfId="17" totalsRowDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I25" headerRowDxfId="25" totalsRowDxfId="24">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="38">
+    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="15">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="37">
+    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="14">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="36">
+    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="13">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="12" totalsRowDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="11" totalsRowDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="10" totalsRowDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="9" totalsRowDxfId="35">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1492,7 +1536,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="34"/>
     <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{1CC9D42E-8B8D-4781-B4E6-7B024D0D4DB5}" name="pri-1-10"/>
   </tableColumns>
@@ -2150,19 +2194,141 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
+      <c r="A22" s="6">
+        <f>ROW()-21</f>
+        <v>1</v>
+      </c>
+      <c r="B22" s="6">
+        <v>10</v>
+      </c>
+      <c r="C22" s="6" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</f>
+        <v>10.11.0.2</v>
+      </c>
+      <c r="D22" s="6" t="str">
+        <f>$E$5</f>
+        <v>10.11.0.1</v>
+      </c>
+      <c r="E22" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F22" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="G22" s="11">
+        <v>4</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I22" s="11">
+        <f>$G22-3</f>
+        <v>1</v>
+      </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <f>ROW()-21</f>
+        <v>2</v>
+      </c>
+      <c r="B23" s="6">
+        <v>10</v>
+      </c>
+      <c r="C23" s="16" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A23)</f>
+        <v>10.11.0.3</v>
+      </c>
+      <c r="D23" s="16" t="str">
+        <f>$E$5</f>
+        <v>10.11.0.1</v>
+      </c>
+      <c r="E23" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="G23" s="11">
+        <v>4</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" s="17">
+        <f>$G23-3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6">
+        <f>ROW()-21</f>
+        <v>3</v>
+      </c>
+      <c r="B24" s="6">
+        <v>10</v>
+      </c>
+      <c r="C24" s="16" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A24)</f>
+        <v>10.11.0.4</v>
+      </c>
+      <c r="D24" s="16" t="str">
+        <f>$E$5</f>
+        <v>10.11.0.1</v>
+      </c>
+      <c r="E24" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F24" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="G24" s="11">
+        <v>4</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I24" s="17">
+        <f>$G24-3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="6">
+        <f>ROW()-21</f>
+        <v>4</v>
+      </c>
+      <c r="B25" s="6">
+        <v>10</v>
+      </c>
+      <c r="C25" s="16" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
+        <v>10.11.0.5</v>
+      </c>
+      <c r="D25" s="16" t="str">
+        <f>$E$5</f>
+        <v>10.11.0.1</v>
+      </c>
+      <c r="E25" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F25" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="G25" s="11">
+        <v>4</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" s="17">
+        <f>$G25-3</f>
+        <v>1</v>
+      </c>
+    </row>
     <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3141,7 +3307,7 @@
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22" xr:uid="{E30D0828-D6F0-4F57-98C2-21AEB5B698E8}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22:F25" xr:uid="{D03F78DE-2965-48F5-B2E0-691EFE7B1D70}">
       <formula1>IF(F22="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(F22,"-"),"."))&lt;=$G22-3)</formula1>
     </dataValidation>
   </dataValidations>
@@ -3598,6 +3764,7 @@
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
+        <f>ROW()-21</f>
         <v>1</v>
       </c>
       <c r="B22" s="6">
@@ -3615,22 +3782,88 @@
         <f>$F$5</f>
         <v>255.255.0.0</v>
       </c>
-      <c r="F22" s="6">
-        <v>30.1</v>
+      <c r="F22" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="G22" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>46</v>
       </c>
       <c r="I22" s="11">
         <f>$G22-3</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="23" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6">
+        <f>ROW()-21</f>
+        <v>2</v>
+      </c>
+      <c r="B23" s="6">
+        <v>10</v>
+      </c>
+      <c r="C23" s="16" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A23)</f>
+        <v>10.12.0.3</v>
+      </c>
+      <c r="D23" s="16" t="str">
+        <f>$E$5</f>
+        <v>10.12.0.1</v>
+      </c>
+      <c r="E23" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" s="11">
+        <v>10</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I23" s="17">
+        <f>$G23-3</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6">
+        <f>ROW()-21</f>
+        <v>3</v>
+      </c>
+      <c r="B24" s="6">
+        <v>10</v>
+      </c>
+      <c r="C24" s="16" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A24)</f>
+        <v>10.12.0.4</v>
+      </c>
+      <c r="D24" s="16" t="str">
+        <f>$E$5</f>
+        <v>10.12.0.1</v>
+      </c>
+      <c r="E24" s="6" t="str">
+        <f>$F$5</f>
+        <v>255.255.0.0</v>
+      </c>
+      <c r="F24" s="6">
+        <v>30.17</v>
+      </c>
+      <c r="G24" s="11">
+        <v>20</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I24" s="17">
+        <f>$G24-3</f>
+        <v>17</v>
+      </c>
+    </row>
     <row r="25" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4603,7 +4836,7 @@
     <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22" xr:uid="{95DCB370-0280-4896-A3B5-1510F9D5C323}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F22:F24" xr:uid="{755C67B3-35A1-41CF-AFAD-859DFFCA6014}">
       <formula1>IF(F22="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(F22,"-"),"."))&lt;=$G22-3)</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
port no sh add
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575F4A5D-A441-4C0F-800A-E462E8EED511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E19B13-2439-4A0C-B471-D027FC47DA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -282,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -325,18 +325,15 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="111">
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
@@ -344,16 +341,25 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -394,11 +400,10 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -414,77 +419,9 @@
     </dxf>
     <dxf>
       <font>
-        <sz val="11"/>
+        <color theme="1"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -496,10 +433,28 @@
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -523,10 +478,11 @@
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -538,49 +494,87 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color theme="1"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1383,39 +1377,39 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="33" dataDxfId="32" totalsRowDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="45" dataDxfId="44" totalsRowDxfId="43">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="42">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="39" totalsRowDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I24" headerRowDxfId="23" totalsRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I24" headerRowDxfId="37" totalsRowDxfId="36">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="35">
       <calculatedColumnFormula>ROW()-21</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="33">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="32">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="31">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="3" totalsRowDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="2" totalsRowDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="1" totalsRowDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="0" totalsRowDxfId="18">
+    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="28" totalsRowDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="26" totalsRowDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="24" totalsRowDxfId="23">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1434,7 +1428,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="22"/>
     <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{BBB41126-CDAD-40BD-92C3-0A8EEC64127E}" name="pri-1-10"/>
   </tableColumns>
@@ -1473,37 +1467,37 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="45" dataDxfId="44" totalsRowDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="21" dataDxfId="20" totalsRowDxfId="19">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="42">
+    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="18">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I25" headerRowDxfId="25" totalsRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I25" headerRowDxfId="14" totalsRowDxfId="13">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="10">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="14">
+    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="9">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="13">
+    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="8">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="12" totalsRowDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="11" totalsRowDxfId="37"/>
-    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="10" totalsRowDxfId="36"/>
-    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="9" totalsRowDxfId="35">
+    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1536,7 +1530,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="46"/>
     <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{1CC9D42E-8B8D-4781-B4E6-7B024D0D4DB5}" name="pri-1-10"/>
   </tableColumns>
@@ -2235,11 +2229,11 @@
       <c r="B23" s="6">
         <v>10</v>
       </c>
-      <c r="C23" s="16" t="str">
+      <c r="C23" s="6" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A23)</f>
         <v>10.11.0.3</v>
       </c>
-      <c r="D23" s="16" t="str">
+      <c r="D23" s="6" t="str">
         <f>$E$5</f>
         <v>10.11.0.1</v>
       </c>
@@ -2256,7 +2250,7 @@
       <c r="H23" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="11">
         <f>$G23-3</f>
         <v>1</v>
       </c>
@@ -2269,11 +2263,11 @@
       <c r="B24" s="6">
         <v>10</v>
       </c>
-      <c r="C24" s="16" t="str">
+      <c r="C24" s="6" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A24)</f>
         <v>10.11.0.4</v>
       </c>
-      <c r="D24" s="16" t="str">
+      <c r="D24" s="6" t="str">
         <f>$E$5</f>
         <v>10.11.0.1</v>
       </c>
@@ -2290,7 +2284,7 @@
       <c r="H24" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I24" s="17">
+      <c r="I24" s="11">
         <f>$G24-3</f>
         <v>1</v>
       </c>
@@ -2303,11 +2297,11 @@
       <c r="B25" s="6">
         <v>10</v>
       </c>
-      <c r="C25" s="16" t="str">
+      <c r="C25" s="6" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
         <v>10.11.0.5</v>
       </c>
-      <c r="D25" s="16" t="str">
+      <c r="D25" s="6" t="str">
         <f>$E$5</f>
         <v>10.11.0.1</v>
       </c>
@@ -2324,7 +2318,7 @@
       <c r="H25" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I25" s="17">
+      <c r="I25" s="11">
         <f>$G25-3</f>
         <v>1</v>
       </c>
@@ -3804,11 +3798,11 @@
       <c r="B23" s="6">
         <v>10</v>
       </c>
-      <c r="C23" s="16" t="str">
+      <c r="C23" s="6" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A23)</f>
         <v>10.12.0.3</v>
       </c>
-      <c r="D23" s="16" t="str">
+      <c r="D23" s="6" t="str">
         <f>$E$5</f>
         <v>10.12.0.1</v>
       </c>
@@ -3825,7 +3819,7 @@
       <c r="H23" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I23" s="17">
+      <c r="I23" s="11">
         <f>$G23-3</f>
         <v>7</v>
       </c>
@@ -3838,11 +3832,11 @@
       <c r="B24" s="6">
         <v>10</v>
       </c>
-      <c r="C24" s="16" t="str">
+      <c r="C24" s="6" t="str">
         <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A24)</f>
         <v>10.12.0.4</v>
       </c>
-      <c r="D24" s="16" t="str">
+      <c r="D24" s="6" t="str">
         <f>$E$5</f>
         <v>10.12.0.1</v>
       </c>
@@ -3851,7 +3845,7 @@
         <v>255.255.0.0</v>
       </c>
       <c r="F24" s="6">
-        <v>30.17</v>
+        <v>30.1</v>
       </c>
       <c r="G24" s="11">
         <v>20</v>
@@ -3859,7 +3853,7 @@
       <c r="H24" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I24" s="17">
+      <c r="I24" s="11">
         <f>$G24-3</f>
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
added hashed pass insted
</commit_message>
<xml_diff>
--- a/demo.xlsx
+++ b/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D2BFBB-20F5-4993-BD44-26EF119EB636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7511A592-264A-48D3-A91D-D72E2E5CAFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="50">
   <si>
     <t>site</t>
   </si>
@@ -57,9 +57,6 @@
     <t>admin</t>
   </si>
   <si>
-    <t>cisco</t>
-  </si>
-  <si>
     <t>0 - 4</t>
   </si>
   <si>
@@ -181,6 +178,12 @@
   </si>
   <si>
     <t>pri-afxx</t>
+  </si>
+  <si>
+    <t>secret</t>
+  </si>
+  <si>
+    <t>$9$0nNdTjfcaOQFlP$4VgON16XmZXlfGr4BcOzEN7OoRxfPIAcXDQ0afwx67k</t>
   </si>
 </sst>
 </file>
@@ -323,7 +326,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="111">
+  <dxfs count="117">
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -398,6 +401,159 @@
     </dxf>
     <dxf>
       <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -469,108 +625,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -581,12 +635,12 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
+        <sz val="10"/>
+        <color theme="1"/>
         <name val="Arial"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -1231,100 +1285,100 @@
   </dxfs>
   <tableStyles count="16">
     <tableStyle name="Site 1 (HUB)-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="110"/>
-      <tableStyleElement type="headerRow" dxfId="109"/>
-      <tableStyleElement type="firstRowStripe" dxfId="108"/>
-      <tableStyleElement type="secondRowStripe" dxfId="107"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="116"/>
+      <tableStyleElement type="headerRow" dxfId="115"/>
+      <tableStyleElement type="firstRowStripe" dxfId="114"/>
+      <tableStyleElement type="secondRowStripe" dxfId="113"/>
     </tableStyle>
     <tableStyle name="Site 3-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="106"/>
-      <tableStyleElement type="headerRow" dxfId="105"/>
-      <tableStyleElement type="firstRowStripe" dxfId="104"/>
-      <tableStyleElement type="secondRowStripe" dxfId="103"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="112"/>
+      <tableStyleElement type="headerRow" dxfId="111"/>
+      <tableStyleElement type="firstRowStripe" dxfId="110"/>
+      <tableStyleElement type="secondRowStripe" dxfId="109"/>
     </tableStyle>
     <tableStyle name="Site 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="102"/>
-      <tableStyleElement type="headerRow" dxfId="101"/>
-      <tableStyleElement type="firstRowStripe" dxfId="100"/>
-      <tableStyleElement type="secondRowStripe" dxfId="99"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="108"/>
+      <tableStyleElement type="headerRow" dxfId="107"/>
+      <tableStyleElement type="firstRowStripe" dxfId="106"/>
+      <tableStyleElement type="secondRowStripe" dxfId="105"/>
     </tableStyle>
     <tableStyle name="Site 4-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="98"/>
-      <tableStyleElement type="headerRow" dxfId="97"/>
-      <tableStyleElement type="firstRowStripe" dxfId="96"/>
-      <tableStyleElement type="secondRowStripe" dxfId="95"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="104"/>
+      <tableStyleElement type="headerRow" dxfId="103"/>
+      <tableStyleElement type="firstRowStripe" dxfId="102"/>
+      <tableStyleElement type="secondRowStripe" dxfId="101"/>
     </tableStyle>
     <tableStyle name="Site 3-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="94"/>
-      <tableStyleElement type="headerRow" dxfId="93"/>
-      <tableStyleElement type="firstRowStripe" dxfId="92"/>
-      <tableStyleElement type="secondRowStripe" dxfId="91"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="100"/>
+      <tableStyleElement type="headerRow" dxfId="99"/>
+      <tableStyleElement type="firstRowStripe" dxfId="98"/>
+      <tableStyleElement type="secondRowStripe" dxfId="97"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="90"/>
-      <tableStyleElement type="headerRow" dxfId="89"/>
-      <tableStyleElement type="firstRowStripe" dxfId="88"/>
-      <tableStyleElement type="secondRowStripe" dxfId="87"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="96"/>
+      <tableStyleElement type="headerRow" dxfId="95"/>
+      <tableStyleElement type="firstRowStripe" dxfId="94"/>
+      <tableStyleElement type="secondRowStripe" dxfId="93"/>
     </tableStyle>
     <tableStyle name="Site 2-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="86"/>
-      <tableStyleElement type="headerRow" dxfId="85"/>
-      <tableStyleElement type="firstRowStripe" dxfId="84"/>
-      <tableStyleElement type="secondRowStripe" dxfId="83"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="92"/>
+      <tableStyleElement type="headerRow" dxfId="91"/>
+      <tableStyleElement type="firstRowStripe" dxfId="90"/>
+      <tableStyleElement type="secondRowStripe" dxfId="89"/>
     </tableStyle>
     <tableStyle name="Site 3-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="82"/>
-      <tableStyleElement type="headerRow" dxfId="81"/>
-      <tableStyleElement type="firstRowStripe" dxfId="80"/>
-      <tableStyleElement type="secondRowStripe" dxfId="79"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="88"/>
+      <tableStyleElement type="headerRow" dxfId="87"/>
+      <tableStyleElement type="firstRowStripe" dxfId="86"/>
+      <tableStyleElement type="secondRowStripe" dxfId="85"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF08000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="78"/>
-      <tableStyleElement type="headerRow" dxfId="77"/>
-      <tableStyleElement type="firstRowStripe" dxfId="76"/>
-      <tableStyleElement type="secondRowStripe" dxfId="75"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="84"/>
+      <tableStyleElement type="headerRow" dxfId="83"/>
+      <tableStyleElement type="firstRowStripe" dxfId="82"/>
+      <tableStyleElement type="secondRowStripe" dxfId="81"/>
     </tableStyle>
     <tableStyle name="Site 4-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF09000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="74"/>
-      <tableStyleElement type="headerRow" dxfId="73"/>
-      <tableStyleElement type="firstRowStripe" dxfId="72"/>
-      <tableStyleElement type="secondRowStripe" dxfId="71"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="80"/>
+      <tableStyleElement type="headerRow" dxfId="79"/>
+      <tableStyleElement type="firstRowStripe" dxfId="78"/>
+      <tableStyleElement type="secondRowStripe" dxfId="77"/>
     </tableStyle>
     <tableStyle name="Site 3-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0A000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="70"/>
-      <tableStyleElement type="headerRow" dxfId="69"/>
-      <tableStyleElement type="firstRowStripe" dxfId="68"/>
-      <tableStyleElement type="secondRowStripe" dxfId="67"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="76"/>
+      <tableStyleElement type="headerRow" dxfId="75"/>
+      <tableStyleElement type="firstRowStripe" dxfId="74"/>
+      <tableStyleElement type="secondRowStripe" dxfId="73"/>
     </tableStyle>
     <tableStyle name="Site 1 (HUB)-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0B000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="66"/>
-      <tableStyleElement type="headerRow" dxfId="65"/>
-      <tableStyleElement type="firstRowStripe" dxfId="64"/>
-      <tableStyleElement type="secondRowStripe" dxfId="63"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="72"/>
+      <tableStyleElement type="headerRow" dxfId="71"/>
+      <tableStyleElement type="firstRowStripe" dxfId="70"/>
+      <tableStyleElement type="secondRowStripe" dxfId="69"/>
     </tableStyle>
     <tableStyle name="Site 2-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0C000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="62"/>
-      <tableStyleElement type="headerRow" dxfId="61"/>
-      <tableStyleElement type="firstRowStripe" dxfId="60"/>
-      <tableStyleElement type="secondRowStripe" dxfId="59"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="68"/>
+      <tableStyleElement type="headerRow" dxfId="67"/>
+      <tableStyleElement type="firstRowStripe" dxfId="66"/>
+      <tableStyleElement type="secondRowStripe" dxfId="65"/>
     </tableStyle>
     <tableStyle name="Site 4-style 3" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0D000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="58"/>
-      <tableStyleElement type="headerRow" dxfId="57"/>
-      <tableStyleElement type="firstRowStripe" dxfId="56"/>
-      <tableStyleElement type="secondRowStripe" dxfId="55"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="64"/>
+      <tableStyleElement type="headerRow" dxfId="63"/>
+      <tableStyleElement type="firstRowStripe" dxfId="62"/>
+      <tableStyleElement type="secondRowStripe" dxfId="61"/>
     </tableStyle>
     <tableStyle name="Site 2-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0E000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="54"/>
-      <tableStyleElement type="headerRow" dxfId="53"/>
-      <tableStyleElement type="firstRowStripe" dxfId="52"/>
-      <tableStyleElement type="secondRowStripe" dxfId="51"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="60"/>
+      <tableStyleElement type="headerRow" dxfId="59"/>
+      <tableStyleElement type="firstRowStripe" dxfId="58"/>
+      <tableStyleElement type="secondRowStripe" dxfId="57"/>
     </tableStyle>
     <tableStyle name="Site 4-style 4" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF0F000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="50"/>
-      <tableStyleElement type="headerRow" dxfId="49"/>
-      <tableStyleElement type="firstRowStripe" dxfId="48"/>
-      <tableStyleElement type="secondRowStripe" dxfId="47"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="56"/>
+      <tableStyleElement type="headerRow" dxfId="55"/>
+      <tableStyleElement type="firstRowStripe" dxfId="54"/>
+      <tableStyleElement type="secondRowStripe" dxfId="53"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1339,14 +1393,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:F2">
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabell5" displayName="Tabell5" ref="A1:G2">
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="site"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="intf_prefix"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="router-id"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
+    <tableColumn id="7" xr3:uid="{754ADF79-920D-4601-911B-DB20F4E9EEB9}" name="secret" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="Site 1 (HUB)-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1371,39 +1426,40 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:D19" headerRowDxfId="45" dataDxfId="44" totalsRowDxfId="43">
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{EA312CD4-9955-4DBC-87B3-6D788BE89D2E}" name="Tabell13192530" displayName="Tabell13192530" ref="A18:E19" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{FCAD462F-C9DE-45E3-B342-8BC685D1666E}" name="site" dataDxfId="21">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{A37D0432-8751-44ED-8106-422243C1F04B}" name="brukernavn" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{1A9A17E0-8442-4E89-96DC-BC0A8BECBBCA}" name="passord" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{F0C81F5E-B27A-43FB-83C1-1FEB580854DE}" name="vty_lines" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{E8DA5B0D-4B09-4D1E-BDAB-BAC231407C4D}" name="secret" dataDxfId="16" totalsRowDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I22" headerRowDxfId="37" totalsRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1746730A-1530-4A6C-8C70-0F2C6BF9753C}" name="Tabell161824282" displayName="Tabell161824282" ref="A21:I22" headerRowDxfId="14" totalsRowDxfId="13">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="35">
+    <tableColumn id="1" xr3:uid="{15F3A197-501D-4FB4-9993-D97C276F45D1}" name="SW" dataDxfId="12">
       <calculatedColumnFormula>ROW()-21</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="33">
+    <tableColumn id="2" xr3:uid="{74DD496A-588F-4B13-B651-6375E15475E0}" name="MGMT Vlan" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{DADAFDFC-5D9A-4BEF-83FF-73C8B73914A7}" name="MGMT ip" dataDxfId="10">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="32">
+    <tableColumn id="4" xr3:uid="{42D46B63-EECB-4A1E-9799-D2E7774B9BCD}" name="gateway" dataDxfId="9">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="31">
+    <tableColumn id="5" xr3:uid="{0BA7E9B1-43B9-44A7-AEF2-587DFD6DB8EE}" name="mask" dataDxfId="8">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="30" totalsRowDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="26" totalsRowDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="24" totalsRowDxfId="23">
+    <tableColumn id="6" xr3:uid="{5B7AA8BC-D315-4E8D-8528-C2AE65848FDF}" name="vlan-antall" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{1088FF3C-FB1C-4E78-BE34-551D9AC36C3C}" name="num_ports" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{19FD676B-E225-4461-8031-718593F85D50}" name="intf_prefix" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{B26584E6-2A20-4139-9852-FBB25CD74431}" name="num_port_ledig" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1422,7 +1478,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{CE1C3544-35AB-45BD-B168-A59522955D24}" name="antall-res" dataDxfId="51"/>
     <tableColumn id="10" xr3:uid="{5AE4CD65-C2FF-447E-B037-873FB4F36B65}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{BBB41126-CDAD-40BD-92C3-0A8EEC64127E}" name="pri-1-10"/>
   </tableColumns>
@@ -1461,37 +1517,38 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:D19" headerRowDxfId="21" dataDxfId="20" totalsRowDxfId="19">
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{D9D18493-1508-418F-A690-377066CBE6D1}" name="Tabell131921" displayName="Tabell131921" ref="A18:E19" headerRowDxfId="50" dataDxfId="49" totalsRowDxfId="48">
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{2906F324-3A93-4FB9-9A3C-D48E0E017DE1}" name="site" dataDxfId="47">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{EACB8E41-CE14-43F2-9E46-F1D9E473C840}" name="brukernavn" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{BDD570DD-38B1-4E0D-8E69-41BC5527F423}" name="passord" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{0C9E5C25-E441-46FF-92BD-E2BEA9C8A2C6}" name="vty_lines" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{E15E69AB-85DA-4C56-B495-1EB315268322}" name="secret" dataDxfId="43" totalsRowDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="Site 4-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" insertRow="1" headerRowDxfId="14" totalsRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{80770F74-6AF8-4ED1-9361-404458E55511}" name="Tabell16182428" displayName="Tabell16182428" ref="A21:I22" insertRow="1" headerRowDxfId="41" totalsRowDxfId="40">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="10">
+    <tableColumn id="1" xr3:uid="{1B73E0C7-C498-41F8-BAC8-7E845E00CB65}" name="SW" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{55746631-7369-4BB6-92AF-BC912FBA9E5B}" name="MGMT Vlan" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{33D1D208-4592-452F-9EE7-3DD24275FDDC}" name="MGMT ip" dataDxfId="37">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A22)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="9">
+    <tableColumn id="4" xr3:uid="{300ED09A-B325-432A-824C-60A4545FEF10}" name="gateway" dataDxfId="36">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="8">
+    <tableColumn id="5" xr3:uid="{DE41E3AD-2DD4-4E00-AAA7-E16DA0B7B327}" name="mask" dataDxfId="35">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="1" totalsRowDxfId="0">
+    <tableColumn id="6" xr3:uid="{10A4DA4A-2584-4B29-9285-F3E796366BC6}" name="vlan-antall" dataDxfId="34" totalsRowDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{40A0DCDD-4793-4C04-AB5A-E199F256A0D9}" name="num_ports" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{D6B9E8CD-F7E4-4AF1-8D5B-45A78B5D62E7}" name="intf_prefix" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{03637906-AC3E-4DB7-AEDB-025CDAD6ADBA}" name="num_port_ledig" dataDxfId="28" totalsRowDxfId="27">
       <calculatedColumnFormula>$G22-3</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1500,14 +1557,15 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell1" displayName="Tabell1" ref="A1:F2">
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell1" displayName="Tabell1" ref="A1:G2">
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="intf_prefix"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="router-id"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="vty_lines"/>
+    <tableColumn id="7" xr3:uid="{AB00FC62-D408-4EC3-87DF-1FBB1D6A67CC}" name="secret" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="Site 2-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1524,7 +1582,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{FD71411A-F46A-4E62-B3D3-4B0E2ED5C489}" name="antall-res" dataDxfId="25"/>
     <tableColumn id="10" xr3:uid="{10BC51DC-9FCC-48A1-8D71-0913AE61C798}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{1CC9D42E-8B8D-4781-B4E6-7B024D0D4DB5}" name="pri-1-10"/>
   </tableColumns>
@@ -1775,13 +1833,16 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="2" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</f>
@@ -1791,10 +1852,13 @@
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>8</v>
+      <c r="G2" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1809,42 +1873,42 @@
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>16</v>
-      </c>
       <c r="I4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="K4" s="14" t="s">
         <v>39</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="7">
         <v>10</v>
@@ -1861,7 +1925,7 @@
         <v>10.11.0.1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G5" s="6" t="str">
         <f t="shared" ref="G5:G7" si="1">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
@@ -1883,7 +1947,7 @@
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="7">
         <v>20</v>
@@ -1900,7 +1964,7 @@
         <v>10.21.0.1</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G6" s="6" t="str">
         <f t="shared" si="1"/>
@@ -1922,7 +1986,7 @@
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="7">
         <v>30</v>
@@ -1939,7 +2003,7 @@
         <v>10.31.0.1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G7" s="6" t="str">
         <f t="shared" si="1"/>
@@ -1965,24 +2029,24 @@
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="6">
         <v>10</v>
@@ -1994,10 +2058,10 @@
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="6">
         <v>20</v>
@@ -2009,10 +2073,10 @@
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="6">
         <v>30</v>
@@ -2025,49 +2089,49 @@
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="H14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="6" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H15+A2)</f>
         <v>172.16.0.11</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E15" s="6" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;H15</f>
@@ -2075,7 +2139,7 @@
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H15" s="2">
         <v>10</v>
@@ -2085,17 +2149,17 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="6" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H16+A2)</f>
         <v>172.16.0.31</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E16" s="6" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;H16</f>
@@ -2103,7 +2167,7 @@
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H16" s="2">
         <v>30</v>
@@ -2135,6 +2199,9 @@
       <c r="D18" s="10" t="s">
         <v>5</v>
       </c>
+      <c r="E18" s="10" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11">
@@ -2145,40 +2212,43 @@
         <v>6</v>
       </c>
       <c r="C19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="11" t="s">
-        <v>8</v>
+      <c r="E19" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F21" s="5" t="s">
+      <c r="G21" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>45</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>1</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3226,13 +3296,16 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="2" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</f>
@@ -3242,10 +3315,13 @@
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>8</v>
+      <c r="G2" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3260,42 +3336,42 @@
     </row>
     <row r="4" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="H4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="I4" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="K4" s="14" t="s">
         <v>39</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="7">
         <v>10</v>
@@ -3312,7 +3388,7 @@
         <v>10.12.0.1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G5" s="6" t="str">
         <f t="shared" ref="G5:G7" si="1">LEFT(D5,LEN(D5)-1)&amp;"1"</f>
@@ -3334,7 +3410,7 @@
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="7">
         <v>20</v>
@@ -3351,7 +3427,7 @@
         <v>10.22.0.1</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G6" s="6" t="str">
         <f t="shared" si="1"/>
@@ -3373,7 +3449,7 @@
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="7">
         <v>30</v>
@@ -3390,7 +3466,7 @@
         <v>10.32.0.1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G7" s="6" t="str">
         <f t="shared" si="1"/>
@@ -3416,24 +3492,24 @@
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="6">
         <v>10</v>
@@ -3445,10 +3521,10 @@
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11" s="6">
         <v>20</v>
@@ -3460,10 +3536,10 @@
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12" s="6">
         <v>30</v>
@@ -3476,49 +3552,49 @@
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="G14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="H14" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="I14" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="J14" s="13" t="s">
         <v>33</v>
-      </c>
-      <c r="J14" s="13" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="6" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H15+A2)</f>
         <v>172.16.0.12</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E15" s="6" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;H15</f>
@@ -3526,7 +3602,7 @@
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H15" s="2">
         <v>10</v>
@@ -3539,17 +3615,17 @@
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="6" t="str">
         <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H16+A2)</f>
         <v>172.16.0.32</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E16" s="6" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;H16</f>
@@ -3557,7 +3633,7 @@
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H16" s="2">
         <v>30</v>
@@ -3582,6 +3658,9 @@
       <c r="D18" s="10" t="s">
         <v>5</v>
       </c>
+      <c r="E18" s="10" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11">
@@ -3592,40 +3671,43 @@
         <v>6</v>
       </c>
       <c r="C19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="11" t="s">
-        <v>8</v>
+      <c r="E19" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="21" spans="1:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F21" s="5" t="s">
+      <c r="G21" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>45</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>1</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3655,7 +3737,7 @@
         <v>4</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I22" s="11">
         <f>$G22-3</f>

</xml_diff>